<commit_message>
refactor: remove unused scheduler_config from seeding
- Skip scheduler_config (not in use - too complex)
- Keep only essential data: users, obat, kategori, email_config
- Clean seeding process for deployment
- Update export script to skip scheduler config
</commit_message>
<xml_diff>
--- a/seed_data.xlsx
+++ b/seed_data.xlsx
@@ -3486,39 +3486,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>config_type</v>
-      </c>
-      <c r="B1" t="str">
-        <v>interval_hari</v>
-      </c>
-      <c r="C1" t="str">
-        <v>enabled</v>
-      </c>
-      <c r="D1" t="str">
-        <v>email_jam</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ved_fefo_email</v>
-      </c>
-      <c r="B2">
-        <v>8</v>
-      </c>
-      <c r="C2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D2" t="str">
-        <v>08:30</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>